<commit_message>
add registration app for front end
</commit_message>
<xml_diff>
--- a/outputs/1786501092_BOM.xlsx
+++ b/outputs/1786501092_BOM.xlsx
@@ -14252,51 +14252,43 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>156220-01</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>156220-01</t>
-        </is>
-      </c>
+          <t>156238-01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FAIRING ASSY, MOTOR MOUNT, LWR, INBD, LH</t>
+          <t>FAIRINGASSY,MOTORMOUNT,LWR,INBD,RH</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>BLXWFA000W2U (x1)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>156238-01</t>
+          <t>156228-01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>FAIRINGASSY,MOTORMOUNT,LWR,INBD,RH</t>
+          <t>FAIRINGASSY,MOTORMOUNT,MID,UPR,LH</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -14320,13 +14312,13 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>156228-01</t>
+          <t>156224-01</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>FAIRINGASSY,MOTORMOUNT,MID,UPR,LH</t>
+          <t>FAIRINGASSY,MOTORMOUNT,MID,UPR,RH</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -14350,13 +14342,13 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>156224-01</t>
+          <t>153336-02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>FAIRINGASSY,MOTORMOUNT,MID,UPR,RH</t>
+          <t>FUSELAGEASSY,FWD</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -14380,51 +14372,43 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>148234-01</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>148234-01</t>
-        </is>
-      </c>
+          <t>156217-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LATCH, PUSH-PULL, 0.37" BOLT PROJECTION</t>
+          <t>FAIRING,MOTORMOUNT,LWR,OUTBD,RH</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>BL0000001517 (x2)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>153336-02</t>
+          <t>156227-01</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>FUSELAGEASSY,FWD</t>
+          <t>FAIRING,MOTORMOUNT,MID,LWR,LH</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -14448,60 +14432,52 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>156232-01</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>156232-01</t>
-        </is>
-      </c>
+          <t>156223-01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>FAIRING ASSY, MOTOR MOUNT, UPR, OUTBD, LH</t>
+          <t>FAIRING,MOTORMOUNT,MID,LWR,RH</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E18" t="n">
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>BLXWFA000W5H (x1)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>156235-01</t>
+          <t>159860-01</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>156235-01</t>
+          <t>159860-01</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>FAIRING ASSY, MOTOR MOUNT, UPR, OUTBD, RH</t>
+          <t>INTEGRATED FAIRING ASSY, UPPER</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -14512,7 +14488,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>BLXWFA0014QL (x1)</t>
+          <t>BS0100008V40</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -14524,22 +14500,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>150498-02</t>
+          <t>150931-01</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>150498-02</t>
+          <t>150931-01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>FAIRING ASSY, WING, LOWER, LH, UPPER SIDE</t>
+          <t>HARNESS AS, BLUE, CAM AFT - MK30-CX-3</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -14550,7 +14526,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>BLXWHF02CF7C (x1)</t>
+          <t>BSXR2A002527</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -14562,22 +14538,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>150500-02</t>
+          <t>150930-02</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>150500-02</t>
+          <t>150930-02</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>FAIRING ASSY, WING, LOWER, RH, UPPER SIDE</t>
+          <t>HARNESS AS, BROWN, AVIO LEFT - MK30-CX-3</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -14588,7 +14564,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>BLXWHF02CF7D (x1)</t>
+          <t>BSXR2A003523</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -14600,22 +14576,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>150517-02</t>
+          <t>150933-01</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>150517-02</t>
+          <t>150933-01</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FAIRING ASSY, WING, UPPER, OUTBD, LH</t>
+          <t>HARNESS AS, GREEN, CAM FWD - MK30-CX-3</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -14626,7 +14602,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>BLXWHF02CF7A (x1)</t>
+          <t>BSXR2A002141</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -14638,22 +14614,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>150515-02</t>
+          <t>150932-01</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>150515-02</t>
+          <t>150932-01</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FAIRING ASSY, WING, UPPER, OUTBD, RH</t>
+          <t>HARNESS AS, PINK, AVIO RIGHT - MK30-CX-3</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -14664,7 +14640,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>BLXWHF029G3V (x1)</t>
+          <t>BSXR2A002183</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -14676,22 +14652,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>152348-01</t>
+          <t>154580-04</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>152348-01</t>
+          <t>154580-04</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FAIRING, AFT ASSY, LH</t>
+          <t>IPC, LEFT, BLK 20, CX-3 2.2.1</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -14702,7 +14678,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>BLXWFA00114N (x1)</t>
+          <t>BSXUFAE000E5</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -14714,22 +14690,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>152346-01</t>
+          <t>154581-04</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>152346-01</t>
+          <t>154581-04</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>FAIRING, AFT ASSY, RH</t>
+          <t>IPC, RIGHT, BLK 20, CX-3 2.2.1</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -14740,7 +14716,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>BLXWFA00195F (x1)</t>
+          <t>BSXUFAF000E5</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -14752,22 +14728,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>150298-02</t>
+          <t>156393-02</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>150298-02</t>
+          <t>156393-02</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FAIRING, BATTERY, LH, ASSY</t>
+          <t>CX-3 LIGHTING, ASSY, LH, BLK20</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -14778,7 +14754,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>BLXWFA000XJ0 (x1)</t>
+          <t>BSXUFAG001JC</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -14790,22 +14766,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>150308-02</t>
+          <t>156394-02</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>150308-02</t>
+          <t>156394-02</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>FAIRING, BATTERY, RH, ASSY</t>
+          <t>CX-3 LIGHTING, ASSY, RH, BLK20</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -14816,7 +14792,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>BLXWFA0017SX (x1)</t>
+          <t>BSXUFAH001RR</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -14828,89 +14804,86 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>152350-02</t>
+          <t>147712-03</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>152350-02</t>
+          <t>147712-03</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FAIRING, BOTTOM ASSY</t>
+          <t>LRU, MOTOR, CX-3, IAW</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>BLXWFA001ABD (x1)</t>
+          <t>BSXE00CBM023
+BSXE00CC1006</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>156219-01</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>156219-01</t>
-        </is>
-      </c>
+          <t>161830-01</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FAIRING, MOTOR MOUNT, LWR, OUTBD, LH</t>
+          <t>PLATE,MAIN,FUSELAGE,AFT</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E29" t="n">
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>BLXWFA000V4X (x1)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>156217-01</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
+          <t>159604-01</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>160275-02</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FAIRING,MOTORMOUNT,LWR,OUTBD,RH</t>
+          <t>PROPELLER ASSY, MK30, CENTER, CCW</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -14922,25 +14895,33 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>BSWU01007334</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>156227-01</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
+          <t>159603-01</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>160274-02</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>FAIRING,MOTORMOUNT,MID,LWR,LH</t>
+          <t>PROPELLER ASSY, MK30, CENTER, CW</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -14952,25 +14933,33 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>BSWU01007273</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>156223-01</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
+          <t>159602-01</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>160273-02</t>
+        </is>
+      </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>FAIRING,MOTORMOUNT,MID,LWR,RH</t>
+          <t>PROPELLER ASSY, MK30, OFF-CENTER, CCW</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -14979,48 +14968,54 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>BSWU01007150
+BSWU01007408</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>156231-01</t>
+          <t>159601-01</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>156231-01</t>
+          <t>160272-02</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>FAIRING, MOTOR MOUNT, UPR, INBD, LH</t>
+          <t>PROPELLER ASSY, MK30, OFF-CENTER, CW</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>BLXWFA000W3D (x1)</t>
+          <t>BSWU01007067
+BSWU01007089</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -15032,22 +15027,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>156234-01</t>
+          <t>147080-03</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>156234-01</t>
+          <t>147080-03</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>FAIRING, MOTOR MOUNT, UPR, INBD, RH</t>
+          <t>RANGEFINDER, MK30</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -15058,7 +15053,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>BLXWFA0014Q5 (x1)</t>
+          <t>BSXBG6537048</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -15070,22 +15065,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>152347-01</t>
+          <t>150446-01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>152347-01</t>
+          <t>150446-01</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>FAIRING, SOB ASSY, LH</t>
+          <t>STRUT ASSY, LWR, LH</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -15096,7 +15091,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>BLXWFA000G6S (x1)</t>
+          <t>BSXWFA0009BF</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -15108,55 +15103,43 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>152349-01</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>152349-01</t>
-        </is>
-      </c>
+          <t>150462-01</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>FAIRING, SOB ASSY, RH</t>
+          <t>STRUTASSY,LWR,RH</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E36" t="n">
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>BLXWFA000GWM (x1)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>159860-01</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>159860-01</t>
-        </is>
-      </c>
+          <t>150422-01</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>INTEGRATED FAIRING ASSY, UPPER</t>
+          <t>STRUTASSY,MID,LH</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -15168,114 +15151,94 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>BS0100008V40</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>150509-02</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>150509-02</t>
-        </is>
-      </c>
+          <t>150434-01</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>FAIRING, WING, LOWER, LH, LOWER SIDE</t>
+          <t>STRUTASSY,MID,RH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E38" t="n">
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>BLXWHF02CBFV (x1)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>150510-02</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>150510-02</t>
-        </is>
-      </c>
+          <t>150405-01</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>FAIRING, WING, LOWER, RH, LOWER SIDE</t>
+          <t>STRUTASSY,UPR,LH</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E39" t="n">
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>BLXWHF029ANG (x1)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>150525-02</t>
+          <t>150416-01</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>150525-02</t>
+          <t>150416-01</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>FAIRING, WING, UPPER, INBD, LH</t>
+          <t>STRUT ASSY, UPR, RH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -15286,7 +15249,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>BLXWHF02CBA6 (x1)</t>
+          <t>BSXWFA00094U</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -15298,55 +15261,43 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>150524-02</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>150524-02</t>
-        </is>
-      </c>
+          <t>150364-02</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>FAIRING, WING, UPPER, INBD, RH</t>
+          <t>TRANSMISSIONASSY,PDS</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="E41" t="n">
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>BLXWHF029APK (x1)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>150931-01</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>150931-01</t>
-        </is>
-      </c>
+          <t>160537-01</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>HARNESS AS, BLUE, CAM AFT - MK30-CX-3</t>
+          <t>SKYECHO,ADS-BOUT</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -15358,33 +15309,25 @@
         <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>BSXR2A002527</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>150930-02</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>150930-02</t>
-        </is>
-      </c>
+          <t>159908-01</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>HARNESS AS, BROWN, AVIO LEFT - MK30-CX-3</t>
+          <t>EDDYCURRENTBRAKESYSTEM(ECBS)ASSY</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -15396,33 +15339,25 @@
         <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>BSXR2A003523</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>150933-01</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>150933-01</t>
-        </is>
-      </c>
+          <t>146334-08</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>HARNESS AS, GREEN, CAM FWD - MK30-CX-3</t>
+          <t>ASSY,BATTERY,3.1P</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -15434,38 +15369,34 @@
         <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>BSXR2A002141</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>150932-01</t>
+          <t>156220-01</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>150932-01</t>
+          <t>156220-01</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>HARNESS AS, PINK, AVIO RIGHT - MK30-CX-3</t>
+          <t>FAIRING ASSY, MOTOR MOUNT, LWR, INBD, LH</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -15476,7 +15407,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>BSXR2A002183</t>
+          <t>BLXWFA000W2U (x1)</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -15488,33 +15419,33 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>154580-04</t>
+          <t>148234-01</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>154580-04</t>
+          <t>148234-01</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>IPC, LEFT, BLK 20, CX-3 2.2.1</t>
+          <t>LATCH, PUSH-PULL, 0.37" BOLT PROJECTION</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>BSXUFAE000E5</t>
+          <t>BL0000001517 (x2)</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -15526,22 +15457,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>154581-04</t>
+          <t>156232-01</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>154581-04</t>
+          <t>156232-01</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>IPC, RIGHT, BLK 20, CX-3 2.2.1</t>
+          <t>FAIRING ASSY, MOTOR MOUNT, UPR, OUTBD, LH</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -15552,7 +15483,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>BSXUFAF000E5</t>
+          <t>BLXWFA000W5H (x1)</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -15564,17 +15495,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>156359-01</t>
+          <t>156235-01</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>156359-01</t>
+          <t>156235-01</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>LANDING GEAR, ASSY, WHEEL, SECONDARY</t>
+          <t>FAIRING ASSY, MOTOR MOUNT, UPR, OUTBD, RH</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -15583,41 +15514,41 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F48" t="n">
         <v>1</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>BL01000002X7 (x1)</t>
+          <t>BLXWFA0014QL (x1)</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>NOT SATISFIED</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>156393-02</t>
+          <t>150498-02</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>156393-02</t>
+          <t>150498-02</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CX-3 LIGHTING, ASSY, LH, BLK20</t>
+          <t>FAIRING ASSY, WING, LOWER, LH, UPPER SIDE</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -15628,7 +15559,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>BSXUFAG001JC</t>
+          <t>BLXWHF02CF7C (x1)</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -15640,22 +15571,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>156394-02</t>
+          <t>150500-02</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>156394-02</t>
+          <t>150500-02</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CX-3 LIGHTING, ASSY, RH, BLK20</t>
+          <t>FAIRING ASSY, WING, LOWER, RH, UPPER SIDE</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -15666,7 +15597,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>BSXUFAH001RR</t>
+          <t>BLXWHF02CF7D (x1)</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -15678,56 +15609,55 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>147712-03</t>
+          <t>150517-02</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>147712-03</t>
+          <t>150517-02</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>LRU, MOTOR, CX-3, IAW</t>
+          <t>FAIRING ASSY, WING, UPPER, OUTBD, LH</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>BSXE00CBM023
-BSXE00CC1006</t>
+          <t>BLXWHF02CF7A (x1)</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>NOT SATISFIED</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>152352-02</t>
+          <t>150515-02</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>152352-02</t>
+          <t>150515-02</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>NOSE CONE ASSY</t>
+          <t>FAIRING ASSY, WING, UPPER, OUTBD, RH</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -15743,7 +15673,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>BLXWFA000VET (x1)</t>
+          <t>BLXWHF029G3V (x1)</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -15755,52 +15685,60 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>161830-01</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr"/>
+          <t>152348-01</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>152348-01</t>
+        </is>
+      </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PLATE,MAIN,FUSELAGE,AFT</t>
+          <t>FAIRING, AFT ASSY, LH</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E53" t="n">
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>BLXWFA00114N (x1)</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>159604-01</t>
+          <t>152346-01</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>160275-02</t>
+          <t>152346-01</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>PROPELLER ASSY, MK30, CENTER, CCW</t>
+          <t>FAIRING, AFT ASSY, RH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -15811,7 +15749,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>BSWU01007334</t>
+          <t>BLXWFA00195F (x1)</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -15823,22 +15761,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>159603-01</t>
+          <t>150298-02</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>160274-02</t>
+          <t>150298-02</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PROPELLER ASSY, MK30, CENTER, CW</t>
+          <t>FAIRING, BATTERY, LH, ASSY</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -15849,7 +15787,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>BSWU01007273</t>
+          <t>BLXWFA000XJ0 (x1)</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -15861,34 +15799,33 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>159602-01</t>
+          <t>150308-02</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>160273-02</t>
+          <t>150308-02</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PROPELLER ASSY, MK30, OFF-CENTER, CCW</t>
+          <t>FAIRING, BATTERY, RH, ASSY</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>BSWU01007150
-BSWU01007408</t>
+          <t>BLXWFA0017SX (x1)</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -15900,34 +15837,33 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>159601-01</t>
+          <t>152350-02</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>160272-02</t>
+          <t>152350-02</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>PROPELLER ASSY, MK30, OFF-CENTER, CW</t>
+          <t>FAIRING, BOTTOM ASSY</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>BSWU01007067
-BSWU01007089</t>
+          <t>BLXWFA001ABD (x1)</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -15939,22 +15875,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>147080-03</t>
+          <t>156219-01</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>147080-03</t>
+          <t>156219-01</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>RANGEFINDER, MK30</t>
+          <t>FAIRING, MOTOR MOUNT, LWR, OUTBD, LH</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -15965,7 +15901,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>BSXBG6537048</t>
+          <t>BLXWFA000V4X (x1)</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -15977,17 +15913,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>151009-01</t>
+          <t>156231-01</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>151009-01</t>
+          <t>156231-01</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>SPINNER, MK30, CENTER</t>
+          <t>FAIRING, MOTOR MOUNT, UPR, INBD, LH</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -15996,14 +15932,14 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>BL01000001WQ (x2)</t>
+          <t>BLXWFA000W3D (x1)</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -16015,17 +15951,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>151008-01</t>
+          <t>156234-01</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>151008-01</t>
+          <t>156234-01</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SPINNER, MK30, OFF-CENTER</t>
+          <t>FAIRING, MOTOR MOUNT, UPR, INBD, RH</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -16034,14 +15970,14 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F60" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>BL01000001X5 (x4)</t>
+          <t>BLXWFA0014Q5 (x1)</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -16053,22 +15989,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>150446-01</t>
+          <t>152347-01</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>150446-01</t>
+          <t>152347-01</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>STRUT ASSY, LWR, LH</t>
+          <t>FAIRING, SOB ASSY, LH</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -16079,7 +16015,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>BSXWFA0009BF</t>
+          <t>BLXWFA000G6S (x1)</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -16091,142 +16027,174 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>150462-01</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr"/>
+          <t>152349-01</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>152349-01</t>
+        </is>
+      </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>STRUTASSY,LWR,RH</t>
+          <t>FAIRING, SOB ASSY, RH</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E62" t="n">
         <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>0</v>
-      </c>
-      <c r="G62" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>BLXWFA000GWM (x1)</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>150422-01</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr"/>
+          <t>150509-02</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>150509-02</t>
+        </is>
+      </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>STRUTASSY,MID,LH</t>
+          <t>FAIRING, WING, LOWER, LH, LOWER SIDE</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E63" t="n">
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>0</v>
-      </c>
-      <c r="G63" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>BLXWHF02CBFV (x1)</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>150434-01</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr"/>
+          <t>150510-02</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>150510-02</t>
+        </is>
+      </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>STRUTASSY,MID,RH</t>
+          <t>FAIRING, WING, LOWER, RH, LOWER SIDE</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E64" t="n">
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>0</v>
-      </c>
-      <c r="G64" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>BLXWHF029ANG (x1)</t>
+        </is>
+      </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>150405-01</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr"/>
+          <t>150525-02</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>150525-02</t>
+        </is>
+      </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>STRUTASSY,UPR,LH</t>
+          <t>FAIRING, WING, UPPER, INBD, LH</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E65" t="n">
         <v>1</v>
       </c>
       <c r="F65" t="n">
-        <v>0</v>
-      </c>
-      <c r="G65" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>BLXWHF02CBA6 (x1)</t>
+        </is>
+      </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>150416-01</t>
+          <t>150524-02</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>150416-01</t>
+          <t>150524-02</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>STRUT ASSY, UPR, RH</t>
+          <t>FAIRING, WING, UPPER, INBD, RH</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -16237,7 +16205,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>BSXWFA00094U</t>
+          <t>BLXWHF029APK (x1)</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -16249,47 +16217,55 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>150364-02</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr"/>
+          <t>156359-01</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>156359-01</t>
+        </is>
+      </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>TRANSMISSIONASSY,PDS</t>
+          <t>LANDING GEAR, ASSY, WHEEL, SECONDARY</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E67" t="n">
+        <v>2</v>
+      </c>
+      <c r="F67" t="n">
         <v>1</v>
       </c>
-      <c r="F67" t="n">
-        <v>0</v>
-      </c>
-      <c r="G67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>BL01000002X7 (x1)</t>
+        </is>
+      </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>NOT SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>150503-02</t>
+          <t>152352-02</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>150503-02</t>
+          <t>152352-02</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>WING ASSY, LWR</t>
+          <t>NOSE CONE ASSY</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -16305,7 +16281,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>BLXWFA001940 (x1)</t>
+          <t>BLXWFA000VET (x1)</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -16317,17 +16293,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>150483-02</t>
+          <t>151009-01</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>150483-02</t>
+          <t>151009-01</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>WING ASSY, UPR</t>
+          <t>SPINNER, MK30, CENTER</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -16336,14 +16312,14 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>BLXWFA000TV2 (x1)</t>
+          <t>BL01000001WQ (x2)</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -16355,17 +16331,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>150490-01</t>
+          <t>151008-01</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>150490-01</t>
+          <t>151008-01</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>WINGLET ASSY, LWR, LH</t>
+          <t>SPINNER, MK30, OFF-CENTER</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -16374,14 +16350,14 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F70" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>BLXWFA00144M (x1)</t>
+          <t>BL01000001X5 (x4)</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -16393,17 +16369,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>150494-01</t>
+          <t>150503-02</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>150494-01</t>
+          <t>150503-02</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>WINGLET ASSY, LWR, RH</t>
+          <t>WING ASSY, LWR</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -16419,7 +16395,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>BLXWFA00191V (x1)</t>
+          <t>BLXWFA001940 (x1)</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -16431,17 +16407,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>150479-01</t>
+          <t>150483-02</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>150479-01</t>
+          <t>150483-02</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>WINGLET ASSY, UPR, LH</t>
+          <t>WING ASSY, UPR</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -16457,7 +16433,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>BLXWFA0017PM (x1)</t>
+          <t>BLXWFA000TV2 (x1)</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -16469,17 +16445,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>150475-01</t>
+          <t>150490-01</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>150475-01</t>
+          <t>150490-01</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>WINGLET ASSY, UPR, RH</t>
+          <t>WINGLET ASSY, LWR, LH</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -16495,7 +16471,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>BLXWFA000VQ9 (x1)</t>
+          <t>BLXWFA00144M (x1)</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -16507,90 +16483,114 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>160537-01</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr"/>
+          <t>150494-01</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>150494-01</t>
+        </is>
+      </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SKYECHO,ADS-BOUT</t>
+          <t>WINGLET ASSY, LWR, RH</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E74" t="n">
         <v>1</v>
       </c>
       <c r="F74" t="n">
-        <v>0</v>
-      </c>
-      <c r="G74" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>BLXWFA00191V (x1)</t>
+        </is>
+      </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>159908-01</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr"/>
+          <t>150479-01</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>150479-01</t>
+        </is>
+      </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>EDDYCURRENTBRAKESYSTEM(ECBS)ASSY</t>
+          <t>WINGLET ASSY, UPR, LH</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E75" t="n">
         <v>1</v>
       </c>
       <c r="F75" t="n">
-        <v>0</v>
-      </c>
-      <c r="G75" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>BLXWFA0017PM (x1)</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>146334-08</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr"/>
+          <t>150475-01</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>150475-01</t>
+        </is>
+      </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ASSY,BATTERY,3.1P</t>
+          <t>WINGLET ASSY, UPR, RH</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="E76" t="n">
         <v>1</v>
       </c>
       <c r="F76" t="n">
-        <v>0</v>
-      </c>
-      <c r="G76" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>BLXWFA000VQ9 (x1)</t>
+        </is>
+      </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>SATISFIED</t>
         </is>
       </c>
     </row>
@@ -16724,7 +16724,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BLXWFA000W2U</t>
+          <t>BS0100008V40</t>
         </is>
       </c>
     </row>
@@ -16736,7 +16736,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BL0000001517</t>
+          <t>BSXR2A002527</t>
         </is>
       </c>
     </row>
@@ -16748,7 +16748,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BLXWFA000W5H</t>
+          <t>BSXR2A003523</t>
         </is>
       </c>
     </row>
@@ -16760,7 +16760,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BLXWFA0014QL</t>
+          <t>BSXR2A002141</t>
         </is>
       </c>
     </row>
@@ -16772,7 +16772,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BLXWHF02CF7C</t>
+          <t>BSXR2A002183</t>
         </is>
       </c>
     </row>
@@ -16784,7 +16784,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BLXWHF02CF7D</t>
+          <t>BSXUFAE000E5</t>
         </is>
       </c>
     </row>
@@ -16796,7 +16796,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BLXWHF02CF7A</t>
+          <t>BSXUFAF000E5</t>
         </is>
       </c>
     </row>
@@ -16808,7 +16808,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BLXWHF029G3V</t>
+          <t>BSXUFAG001JC</t>
         </is>
       </c>
     </row>
@@ -16820,7 +16820,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BLXWFA00114N</t>
+          <t>BSXUFAH001RR</t>
         </is>
       </c>
     </row>
@@ -16832,7 +16832,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BLXWFA00195F</t>
+          <t>BSXE00CBM023</t>
         </is>
       </c>
     </row>
@@ -16844,7 +16844,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BLXWFA000XJ0</t>
+          <t>BSXE00CC1006</t>
         </is>
       </c>
     </row>
@@ -16856,7 +16856,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BLXWFA0017SX</t>
+          <t>BSWU01007334</t>
         </is>
       </c>
     </row>
@@ -16868,7 +16868,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BLXWFA001ABD</t>
+          <t>BSWU01007273</t>
         </is>
       </c>
     </row>
@@ -16880,7 +16880,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BLXWFA000V4X</t>
+          <t>BSWU01007150</t>
         </is>
       </c>
     </row>
@@ -16892,7 +16892,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BLXWFA000W3D</t>
+          <t>BSWU01007408</t>
         </is>
       </c>
     </row>
@@ -16904,7 +16904,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BLXWFA0014Q5</t>
+          <t>BSWU01007067</t>
         </is>
       </c>
     </row>
@@ -16916,7 +16916,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BLXWFA000G6S</t>
+          <t>BSWU01007089</t>
         </is>
       </c>
     </row>
@@ -16928,7 +16928,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BLXWFA000GWM</t>
+          <t>BSXBG6537048</t>
         </is>
       </c>
     </row>
@@ -16940,7 +16940,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BS0100008V40</t>
+          <t>BSXWFA0009BF</t>
         </is>
       </c>
     </row>
@@ -16952,7 +16952,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BLXWHF02CBFV</t>
+          <t>BSXWFA00094U</t>
         </is>
       </c>
     </row>
@@ -16964,7 +16964,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BLXWHF029ANG</t>
+          <t>BLXWFA000W2U</t>
         </is>
       </c>
     </row>
@@ -16976,7 +16976,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BLXWHF02CBA6</t>
+          <t>BL0000001517</t>
         </is>
       </c>
     </row>
@@ -16988,7 +16988,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>BLXWHF029APK</t>
+          <t>BLXWFA000W5H</t>
         </is>
       </c>
     </row>
@@ -17000,7 +17000,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>BSXR2A002527</t>
+          <t>BLXWFA0014QL</t>
         </is>
       </c>
     </row>
@@ -17012,7 +17012,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>BSXR2A003523</t>
+          <t>BLXWHF02CF7C</t>
         </is>
       </c>
     </row>
@@ -17024,7 +17024,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>BSXR2A002141</t>
+          <t>BLXWHF02CF7D</t>
         </is>
       </c>
     </row>
@@ -17036,7 +17036,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>BSXR2A002183</t>
+          <t>BLXWHF02CF7A</t>
         </is>
       </c>
     </row>
@@ -17048,7 +17048,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>BSXUFAE000E5</t>
+          <t>BLXWHF029G3V</t>
         </is>
       </c>
     </row>
@@ -17060,7 +17060,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>BSXUFAF000E5</t>
+          <t>BLXWFA00114N</t>
         </is>
       </c>
     </row>
@@ -17072,7 +17072,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>BL01000002X7</t>
+          <t>BLXWFA00195F</t>
         </is>
       </c>
     </row>
@@ -17084,7 +17084,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>BSXUFAG001JC</t>
+          <t>BLXWFA000XJ0</t>
         </is>
       </c>
     </row>
@@ -17096,7 +17096,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BSXUFAH001RR</t>
+          <t>BLXWFA0017SX</t>
         </is>
       </c>
     </row>
@@ -17108,7 +17108,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>BSXE00CBM023</t>
+          <t>BLXWFA001ABD</t>
         </is>
       </c>
     </row>
@@ -17120,7 +17120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>BSXE00CC1006</t>
+          <t>BLXWFA000V4X</t>
         </is>
       </c>
     </row>
@@ -17132,7 +17132,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>BLXWFA000VET</t>
+          <t>BLXWFA000W3D</t>
         </is>
       </c>
     </row>
@@ -17144,7 +17144,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>BSWU01007334</t>
+          <t>BLXWFA0014Q5</t>
         </is>
       </c>
     </row>
@@ -17156,7 +17156,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>BSWU01007273</t>
+          <t>BLXWFA000G6S</t>
         </is>
       </c>
     </row>
@@ -17168,7 +17168,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>BSWU01007150</t>
+          <t>BLXWFA000GWM</t>
         </is>
       </c>
     </row>
@@ -17180,7 +17180,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>BSWU01007408</t>
+          <t>BLXWHF02CBFV</t>
         </is>
       </c>
     </row>
@@ -17192,7 +17192,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>BSWU01007067</t>
+          <t>BLXWHF029ANG</t>
         </is>
       </c>
     </row>
@@ -17204,7 +17204,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>BSWU01007089</t>
+          <t>BLXWHF02CBA6</t>
         </is>
       </c>
     </row>
@@ -17216,7 +17216,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>BSXBG6537048</t>
+          <t>BLXWHF029APK</t>
         </is>
       </c>
     </row>
@@ -17228,7 +17228,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>BL01000001WQ</t>
+          <t>BL01000002X7</t>
         </is>
       </c>
     </row>
@@ -17240,7 +17240,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>BL01000001X5</t>
+          <t>BLXWFA000VET</t>
         </is>
       </c>
     </row>
@@ -17252,7 +17252,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>BSXWFA0009BF</t>
+          <t>BL01000001WQ</t>
         </is>
       </c>
     </row>
@@ -17264,7 +17264,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>BSXWFA00094U</t>
+          <t>BL01000001X5</t>
         </is>
       </c>
     </row>
@@ -17779,28 +17779,28 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>156359-01</t>
+          <t>147712-03</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr"/>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>LANDING GEAR, ASSY, WHEEL, SECONDARY</t>
+          <t>LRU, MOTOR, CX-3, IAW</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="F12" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="1" t="n">
-        <v>1</v>
-      </c>
       <c r="H12" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I12" s="1" t="inlineStr">
         <is>
@@ -17816,13 +17816,13 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>147712-03</t>
+          <t>161830-01</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr"/>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>LRU, MOTOR, CX-3, IAW</t>
+          <t>PLATE,MAIN,FUSELAGE,AFT</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
@@ -17831,17 +17831,17 @@
         </is>
       </c>
       <c r="F13" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H13" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I13" s="1" t="inlineStr">
         <is>
-          <t>NOT SATISFIED</t>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
@@ -17853,13 +17853,13 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>161830-01</t>
+          <t>150462-01</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr"/>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>PLATE,MAIN,FUSELAGE,AFT</t>
+          <t>STRUTASSY,LWR,RH</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr">
@@ -17890,13 +17890,13 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>150462-01</t>
+          <t>150422-01</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr"/>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>STRUTASSY,LWR,RH</t>
+          <t>STRUTASSY,MID,LH</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr">
@@ -17927,13 +17927,13 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>150422-01</t>
+          <t>150434-01</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr"/>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>STRUTASSY,MID,LH</t>
+          <t>STRUTASSY,MID,RH</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr">
@@ -17964,13 +17964,13 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>150434-01</t>
+          <t>150405-01</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr"/>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>STRUTASSY,MID,RH</t>
+          <t>STRUTASSY,UPR,LH</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr">
@@ -18001,13 +18001,13 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>150405-01</t>
+          <t>150364-02</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr"/>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>STRUTASSY,UPR,LH</t>
+          <t>TRANSMISSIONASSY,PDS</t>
         </is>
       </c>
       <c r="E18" s="1" t="inlineStr">
@@ -18038,13 +18038,13 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>150364-02</t>
+          <t>160537-01</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr"/>
       <c r="D19" s="1" t="inlineStr">
         <is>
-          <t>TRANSMISSIONASSY,PDS</t>
+          <t>SKYECHO,ADS-BOUT</t>
         </is>
       </c>
       <c r="E19" s="1" t="inlineStr">
@@ -18075,13 +18075,13 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>160537-01</t>
+          <t>159908-01</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr"/>
       <c r="D20" s="1" t="inlineStr">
         <is>
-          <t>SKYECHO,ADS-BOUT</t>
+          <t>EDDYCURRENTBRAKESYSTEM(ECBS)ASSY</t>
         </is>
       </c>
       <c r="E20" s="1" t="inlineStr">
@@ -18112,13 +18112,13 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>159908-01</t>
+          <t>146334-08</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr"/>
       <c r="D21" s="1" t="inlineStr">
         <is>
-          <t>EDDYCURRENTBRAKESYSTEM(ECBS)ASSY</t>
+          <t>ASSY,BATTERY,3.1P</t>
         </is>
       </c>
       <c r="E21" s="1" t="inlineStr">
@@ -18149,32 +18149,32 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>146334-08</t>
+          <t>156359-01</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr"/>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>ASSY,BATTERY,3.1P</t>
+          <t>LANDING GEAR, ASSY, WHEEL, SECONDARY</t>
         </is>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="F22" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="1" t="n">
         <v>1</v>
-      </c>
-      <c r="G22" s="1" t="n">
-        <v>0</v>
       </c>
       <c r="H22" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I22" s="1" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>NOT SATISFIED</t>
         </is>
       </c>
     </row>

</xml_diff>